<commit_message>
Updated Base Class and Faling TCS
</commit_message>
<xml_diff>
--- a/src/main/java/com/NonKeyword_FutureReadyFramework/automation/config/Config.xlsx
+++ b/src/main/java/com/NonKeyword_FutureReadyFramework/automation/config/Config.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C15964BA-F439-4918-BC7B-D93F791C82CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A699532-0C8E-48A2-B22B-E254F8ABD7CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -488,7 +488,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.8" x14ac:dyDescent="0.4">

</xml_diff>